<commit_message>
OHAP300515C: the Rick Stein's Cookery School fish logo works order replaces the 2000-2020 one
New artwork (the fish), the logo centre bib, finishing pressed, trimmed,
folded for display, tissued and stickered (JH 9/2/26). The thread colour
is not on this sheet; the earlier one had white. The superseded sheet is
kept under works-orders/.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011dreybnjXTET1yVq4copdE
</commit_message>
<xml_diff>
--- a/works-orders/OHAP300515C-RickStein-CookerySchool.xlsx
+++ b/works-orders/OHAP300515C-RickStein-CookerySchool.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Order forms\Oliver Harvey\OH Customers\Rick Stein - Seafood Trading\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB6B9984-1E18-46DE-BA9D-5625023B9F40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE342EF1-DB23-4395-B8AE-CD0071A78415}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="78">
   <si>
     <t xml:space="preserve">DATE ISSUED </t>
   </si>
@@ -87,6 +87,9 @@
     <t xml:space="preserve">ISSUED BY </t>
   </si>
   <si>
+    <t>EMBROIDERY</t>
+  </si>
+  <si>
     <t xml:space="preserve">SALES/RENTAL </t>
   </si>
   <si>
@@ -213,19 +216,19 @@
     <t>YL - Added thread shade - 29.1.19</t>
   </si>
   <si>
-    <t>YL - Added Rick Steins - 2000- 2020 logo. - 23.12.2019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMBROIDERY </t>
-  </si>
-  <si>
-    <t xml:space="preserve">WHITE - CENTRE BIB </t>
-  </si>
-  <si>
     <t xml:space="preserve">  OHAP300515C</t>
   </si>
   <si>
-    <t>jh 23/3/22  corrected care label information</t>
+    <t>Rick Stein's Cookery School Logo - Centre Bib</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jh 23/3/22 Corrected care label information </t>
+  </si>
+  <si>
+    <t>Linzi</t>
+  </si>
+  <si>
+    <t>OHAP300515C</t>
   </si>
   <si>
     <t>CO5015ECO</t>
@@ -234,25 +237,25 @@
     <t>TIAJO</t>
   </si>
   <si>
-    <t>NAVY  100% ORGANIC COTTON  X149ECO-AM303 260GSM</t>
-  </si>
-  <si>
-    <t>1.0M</t>
-  </si>
-  <si>
-    <t>WASH - 100% ORGANIC COTTON  40 degree wash/ Low tumble dry/2 dot iron/P dry clean/ Do not bleach</t>
-  </si>
-  <si>
-    <t>JH 3/6/25 - Amended to Tiajo Eco fabric and up-dated care label</t>
-  </si>
-  <si>
-    <t>PRESS AND TISSUE</t>
-  </si>
-  <si>
-    <t>re-LS 9/2/26 - Go back to Press and Tissue and product sticker- JH amended</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRESSED, TRIMMED, FOLDED  AND TISSUE. PRODUCT STICKER SET TO RIGHT HAND CORNER. </t>
+    <t>WASH - 100% ORGANIC COTTON  40 degree wash/Low tumble dry/Iron 2 dot/Do not bleach/P dry clean</t>
+  </si>
+  <si>
+    <t>JH Amended to tiajo Eco fabric and amended care label</t>
+  </si>
+  <si>
+    <t>1.0m</t>
+  </si>
+  <si>
+    <t>NAVY  100% ORGANIC COTTON 260gsm X149ECO-AM303</t>
+  </si>
+  <si>
+    <t>NEEDS TO BE PRESSED AND TISSUED!!</t>
+  </si>
+  <si>
+    <t>Re- LS - 9/2/26 now needs to be pressed and tissued. JH Amended.</t>
+  </si>
+  <si>
+    <t>PRESSED, TRIMMED AND FOLDED SIDES IN AND BIB UP FOR DISPLAY.  SET IN TISSUE. PRODUCT STICKER SET TO BOTTOM RIGHT HAND CORNER.</t>
   </si>
 </sst>
 </file>
@@ -425,18 +428,19 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="14"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="16"/>
-      <color indexed="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="14"/>
+      <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -449,14 +453,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="29">
+  <borders count="28">
     <border>
       <left/>
       <right/>
@@ -575,6 +573,26 @@
     </border>
     <border>
       <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="medium">
         <color indexed="64"/>
       </right>
@@ -592,43 +610,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -792,7 +773,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
@@ -831,9 +812,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
@@ -850,7 +828,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -873,33 +850,25 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -910,22 +879,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
@@ -934,53 +903,95 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1003,22 +1014,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1209675</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>289275</xdr:rowOff>
+      <xdr:colOff>371475</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>19051</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>398100</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>1180532</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2191553</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>1009651</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
+        <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1034,8 +1045,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3933825" y="3804000"/>
-          <a:ext cx="3065100" cy="891257"/>
+          <a:off x="3095625" y="4067176"/>
+          <a:ext cx="1820078" cy="990600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1337,86 +1348,88 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.28515625" style="3" customWidth="1"/>
     <col min="2" max="2" width="20.5703125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="37.42578125" style="18" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" style="17" customWidth="1"/>
     <col min="4" max="4" width="20.7109375" style="3" customWidth="1"/>
     <col min="5" max="5" width="26.85546875" style="3" customWidth="1"/>
     <col min="6" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="62" t="s">
-        <v>21</v>
-      </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="63" t="s">
-        <v>59</v>
+      <c r="A1" s="58" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="59" t="s">
+        <v>60</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="65"/>
+      <c r="E1" s="61" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="2" spans="1:5" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="43" t="s">
-        <v>30</v>
+      <c r="B2" s="65"/>
+      <c r="C2" s="41" t="s">
+        <v>31</v>
       </c>
       <c r="D2" s="1"/>
-      <c r="E2" s="66"/>
+      <c r="E2" s="62"/>
     </row>
     <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.4">
-      <c r="A3" s="72" t="s">
-        <v>46</v>
-      </c>
-      <c r="B3" s="73"/>
-      <c r="C3" s="67" t="s">
-        <v>25</v>
-      </c>
-      <c r="D3" s="76"/>
-      <c r="E3" s="42"/>
+      <c r="A3" s="68" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="69"/>
+      <c r="C3" s="63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="72"/>
+      <c r="E3" s="40"/>
     </row>
     <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.4">
-      <c r="A4" s="74"/>
-      <c r="B4" s="75"/>
-      <c r="C4" s="68" t="s">
-        <v>47</v>
-      </c>
-      <c r="D4" s="76"/>
-      <c r="E4" s="42"/>
+      <c r="A4" s="70"/>
+      <c r="B4" s="71"/>
+      <c r="C4" s="64" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" s="72"/>
+      <c r="E4" s="40"/>
     </row>
     <row r="5" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="77"/>
-      <c r="B5" s="78"/>
-      <c r="C5" s="79"/>
-      <c r="D5" s="76"/>
-      <c r="E5" s="42"/>
-    </row>
-    <row r="6" spans="1:5" s="8" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="70" t="s">
+      <c r="A5" s="73"/>
+      <c r="B5" s="74"/>
+      <c r="C5" s="75"/>
+      <c r="D5" s="72"/>
+      <c r="E5" s="40"/>
+    </row>
+    <row r="6" spans="1:5" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="71"/>
+      <c r="B6" s="67"/>
       <c r="C6" s="6" t="s">
         <v>1</v>
       </c>
       <c r="D6" s="7"/>
       <c r="E6" s="6"/>
     </row>
-    <row r="7" spans="1:5" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>2</v>
@@ -1426,7 +1439,9 @@
     <row r="8" spans="1:5" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A8" s="11"/>
       <c r="B8" s="12"/>
-      <c r="C8" s="13"/>
+      <c r="C8" s="88" t="s">
+        <v>68</v>
+      </c>
       <c r="D8" s="11"/>
       <c r="E8" s="5"/>
     </row>
@@ -1440,8 +1455,8 @@
     <row r="10" spans="1:5" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" s="11"/>
       <c r="B10" s="5"/>
-      <c r="C10" s="61" t="s">
-        <v>48</v>
+      <c r="C10" s="57" t="s">
+        <v>49</v>
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="5"/>
@@ -1449,441 +1464,462 @@
     <row r="11" spans="1:5" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A11" s="11"/>
       <c r="B11" s="5"/>
-      <c r="C11" s="60" t="s">
-        <v>74</v>
+      <c r="C11" s="103" t="s">
+        <v>75</v>
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
-        <v>45</v>
-      </c>
+      <c r="A12" s="11"/>
       <c r="B12" s="5"/>
-      <c r="C12" s="11"/>
+      <c r="C12" s="110" t="s">
+        <v>46</v>
+      </c>
       <c r="D12" s="11"/>
       <c r="E12" s="5"/>
     </row>
-    <row r="13" spans="1:5" s="14" customFormat="1" ht="116.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="46" t="s">
-        <v>64</v>
-      </c>
-      <c r="B13" s="90" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="99" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="100"/>
+      <c r="C13" s="91"/>
+      <c r="D13" s="91"/>
+      <c r="E13" s="92"/>
+    </row>
+    <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A14" s="101"/>
+      <c r="C14" s="90" t="s">
         <v>65</v>
       </c>
-      <c r="C13" s="87"/>
-      <c r="D13" s="88"/>
-      <c r="E13" s="89"/>
-    </row>
-    <row r="14" spans="1:5" s="14" customFormat="1" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="28"/>
-      <c r="B14" s="28"/>
-      <c r="C14" s="47" t="s">
+      <c r="D14" s="89"/>
+      <c r="E14" s="93"/>
+    </row>
+    <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A15" s="101"/>
+      <c r="C15" s="90"/>
+      <c r="D15" s="89"/>
+      <c r="E15" s="93"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="101"/>
+      <c r="C16" s="89"/>
+      <c r="D16" s="89"/>
+      <c r="E16" s="93"/>
+    </row>
+    <row r="17" spans="1:5" s="13" customFormat="1" ht="96" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="94"/>
+      <c r="B17" s="95"/>
+      <c r="C17" s="96"/>
+      <c r="D17" s="97"/>
+      <c r="E17" s="98"/>
+    </row>
+    <row r="18" spans="1:5" s="13" customFormat="1" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="43"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="D14" s="47"/>
-      <c r="E14" s="48"/>
-    </row>
-    <row r="15" spans="1:5" s="14" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A15" s="21" t="s">
+      <c r="D18" s="43"/>
+      <c r="E18" s="44"/>
+    </row>
+    <row r="19" spans="1:5" s="13" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+      <c r="A19" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+    </row>
+    <row r="20" spans="1:5" s="13" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+      <c r="A20" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="42"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+    </row>
+    <row r="21" spans="1:5" s="13" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="34"/>
+      <c r="E21" s="19"/>
+    </row>
+    <row r="22" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="35" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" s="35"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="36" t="s">
+        <v>6</v>
+      </c>
+      <c r="E22" s="36" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" s="37" t="s">
+        <v>7</v>
+      </c>
+      <c r="B23" s="38" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="38"/>
+      <c r="D23" s="39"/>
+      <c r="E23" s="40"/>
+    </row>
+    <row r="24" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="40" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" t="s">
+        <v>74</v>
+      </c>
+      <c r="C24" s="76"/>
+      <c r="D24" s="77" t="s">
+        <v>69</v>
+      </c>
+      <c r="E24" s="77" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" s="40" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25" t="s">
+        <v>70</v>
+      </c>
+      <c r="C25" s="78"/>
+      <c r="D25" s="40"/>
+      <c r="E25" s="40"/>
+    </row>
+    <row r="26" spans="1:5" s="14" customFormat="1" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="79" t="s">
+        <v>15</v>
+      </c>
+      <c r="B26" s="102" t="s">
+        <v>73</v>
+      </c>
+      <c r="C26" s="80"/>
+      <c r="D26" s="79"/>
+      <c r="E26" s="33"/>
+    </row>
+    <row r="27" spans="1:5" s="14" customFormat="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="B27" s="27"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="30"/>
+    </row>
+    <row r="28" spans="1:5" s="14" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" s="32" t="s">
+        <v>23</v>
+      </c>
+      <c r="C28" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="D28" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="21"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-    </row>
-    <row r="16" spans="1:5" s="14" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A16" s="21" t="s">
+      <c r="E28" s="30"/>
+    </row>
+    <row r="29" spans="1:5" s="14" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A29" s="45" t="s">
+        <v>54</v>
+      </c>
+      <c r="B29" s="46" t="s">
+        <v>55</v>
+      </c>
+      <c r="C29" s="46" t="s">
+        <v>56</v>
+      </c>
+      <c r="D29" s="47" t="s">
+        <v>57</v>
+      </c>
+      <c r="E29" s="48"/>
+    </row>
+    <row r="30" spans="1:5" s="14" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="45"/>
+      <c r="B30" s="46"/>
+      <c r="C30" s="49" t="s">
+        <v>16</v>
+      </c>
+      <c r="D30" s="47"/>
+      <c r="E30" s="48"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" s="81" t="s">
+        <v>17</v>
+      </c>
+      <c r="B31" s="82" t="s">
+        <v>62</v>
+      </c>
+      <c r="C31" s="83"/>
+      <c r="D31" s="84"/>
+      <c r="E31" s="85"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" s="86" t="s">
+        <v>18</v>
+      </c>
+      <c r="B32" s="78" t="s">
+        <v>61</v>
+      </c>
+      <c r="C32" s="78"/>
+      <c r="D32" s="87"/>
+      <c r="E32" s="40"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" s="86"/>
+      <c r="B33" t="s">
+        <v>37</v>
+      </c>
+      <c r="C33" s="78"/>
+      <c r="D33" s="87"/>
+      <c r="E33" s="40"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="86"/>
+      <c r="B34" t="s">
+        <v>71</v>
+      </c>
+      <c r="C34" s="78"/>
+      <c r="D34" s="87"/>
+      <c r="E34" s="40"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" s="86" t="s">
+        <v>30</v>
+      </c>
+      <c r="B35" t="s">
+        <v>44</v>
+      </c>
+      <c r="C35" s="78"/>
+      <c r="D35" s="87"/>
+      <c r="E35" s="40"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" s="86"/>
+      <c r="B36" t="s">
+        <v>39</v>
+      </c>
+      <c r="C36" s="78"/>
+      <c r="D36" s="87"/>
+      <c r="E36" s="40"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" s="86" t="s">
+        <v>40</v>
+      </c>
+      <c r="B37" t="s">
+        <v>45</v>
+      </c>
+      <c r="C37" s="78"/>
+      <c r="D37" s="87"/>
+      <c r="E37" s="40"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" s="86"/>
+      <c r="B38"/>
+      <c r="C38" s="78"/>
+      <c r="D38" s="87"/>
+      <c r="E38" s="40"/>
+    </row>
+    <row r="39" spans="1:5" s="13" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+      <c r="A39" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="B39" s="55"/>
+      <c r="C39" s="55"/>
+      <c r="D39" s="55"/>
+      <c r="E39" s="56"/>
+    </row>
+    <row r="40" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="104" t="s">
+        <v>52</v>
+      </c>
+      <c r="B40" s="78"/>
+      <c r="C40" s="78"/>
+      <c r="D40" s="78"/>
+      <c r="E40" s="105"/>
+    </row>
+    <row r="41" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="104" t="s">
+        <v>58</v>
+      </c>
+      <c r="B41" s="78"/>
+      <c r="C41" s="78"/>
+      <c r="D41" s="78"/>
+      <c r="E41" s="105"/>
+    </row>
+    <row r="42" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="104" t="s">
+        <v>53</v>
+      </c>
+      <c r="B42" s="78"/>
+      <c r="C42" s="78"/>
+      <c r="D42" s="78"/>
+      <c r="E42" s="105"/>
+    </row>
+    <row r="43" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="104" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="44"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-    </row>
-    <row r="17" spans="1:5" s="14" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="21" t="s">
-        <v>42</v>
-      </c>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="21"/>
-    </row>
-    <row r="18" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B18" s="37"/>
-      <c r="C18" s="37"/>
-      <c r="D18" s="38" t="s">
-        <v>6</v>
-      </c>
-      <c r="E18" s="38" t="s">
+      <c r="B43" s="78"/>
+      <c r="C43" s="78"/>
+      <c r="D43" s="78"/>
+      <c r="E43" s="105"/>
+    </row>
+    <row r="44" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="104" t="s">
+        <v>36</v>
+      </c>
+      <c r="B44" s="78"/>
+      <c r="C44" s="78"/>
+      <c r="D44" s="78"/>
+      <c r="E44" s="105"/>
+    </row>
+    <row r="45" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="104" t="s">
+        <v>33</v>
+      </c>
+      <c r="B45" s="78"/>
+      <c r="C45" s="78"/>
+      <c r="D45" s="78"/>
+      <c r="E45" s="105"/>
+    </row>
+    <row r="46" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="104" t="s">
+        <v>34</v>
+      </c>
+      <c r="B46" s="78"/>
+      <c r="C46" s="78"/>
+      <c r="D46" s="78"/>
+      <c r="E46" s="105"/>
+    </row>
+    <row r="47" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="104" t="s">
+        <v>32</v>
+      </c>
+      <c r="B47" s="38"/>
+      <c r="C47" s="78"/>
+      <c r="D47" s="78"/>
+      <c r="E47" s="105"/>
+    </row>
+    <row r="48" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="104" t="s">
+        <v>35</v>
+      </c>
+      <c r="B48" s="38"/>
+      <c r="C48" s="78"/>
+      <c r="D48" s="78"/>
+      <c r="E48" s="105"/>
+    </row>
+    <row r="49" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="106" t="s">
+        <v>12</v>
+      </c>
+      <c r="B49" s="38"/>
+      <c r="C49" s="78"/>
+      <c r="D49" s="78"/>
+      <c r="E49" s="105"/>
+    </row>
+    <row r="50" spans="1:5" s="13" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="107" t="s">
+        <v>77</v>
+      </c>
+      <c r="B50" s="108"/>
+      <c r="C50" s="108"/>
+      <c r="D50" s="108"/>
+      <c r="E50" s="109"/>
+    </row>
+    <row r="51" spans="1:5" s="16" customFormat="1" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="50" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="39" t="s">
-        <v>7</v>
-      </c>
-      <c r="B19" s="40" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" s="40"/>
-      <c r="D19" s="41"/>
-      <c r="E19" s="42"/>
-    </row>
-    <row r="20" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="42" t="s">
-        <v>4</v>
-      </c>
-      <c r="B20" t="s">
-        <v>70</v>
-      </c>
-      <c r="C20" s="80"/>
-      <c r="D20" s="81" t="s">
-        <v>68</v>
-      </c>
-      <c r="E20" s="81" t="s">
+      <c r="B51" s="51"/>
+      <c r="C51" s="51"/>
+      <c r="D51" s="52"/>
+      <c r="E51" s="53"/>
+    </row>
+    <row r="52" spans="1:5" s="16" customFormat="1" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B52" s="20"/>
+      <c r="C52" s="23"/>
+      <c r="D52" s="21"/>
+      <c r="E52" s="22"/>
+    </row>
+    <row r="53" spans="1:5" s="16" customFormat="1" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="B53" s="20"/>
+      <c r="C53" s="24"/>
+      <c r="D53" s="21"/>
+      <c r="E53" s="22"/>
+    </row>
+    <row r="54" spans="1:5" s="16" customFormat="1" ht="18.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="18" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="42" t="s">
-        <v>14</v>
-      </c>
-      <c r="B21" t="s">
-        <v>69</v>
-      </c>
-      <c r="C21" s="82"/>
-      <c r="D21" s="42"/>
-      <c r="E21" s="42"/>
-    </row>
-    <row r="22" spans="1:5" s="15" customFormat="1" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="83" t="s">
-        <v>15</v>
-      </c>
-      <c r="B22" s="91" t="s">
-        <v>71</v>
-      </c>
-      <c r="C22" s="84"/>
-      <c r="D22" s="83"/>
-      <c r="E22" s="35"/>
-    </row>
-    <row r="23" spans="1:5" s="15" customFormat="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="B23" s="29"/>
-      <c r="C23" s="30"/>
-      <c r="D23" s="31"/>
-      <c r="E23" s="32"/>
-    </row>
-    <row r="24" spans="1:5" s="15" customFormat="1" ht="12" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="33" t="s">
-        <v>26</v>
-      </c>
-      <c r="B24" s="34" t="s">
-        <v>22</v>
-      </c>
-      <c r="C24" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="D24" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="E24" s="32"/>
-    </row>
-    <row r="25" spans="1:5" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A25" s="49" t="s">
-        <v>53</v>
-      </c>
-      <c r="B25" s="50" t="s">
-        <v>54</v>
-      </c>
-      <c r="C25" s="50" t="s">
-        <v>55</v>
-      </c>
-      <c r="D25" s="51" t="s">
-        <v>56</v>
-      </c>
-      <c r="E25" s="52"/>
-    </row>
-    <row r="26" spans="1:5" s="15" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="49"/>
-      <c r="B26" s="50"/>
-      <c r="C26" s="53" t="s">
-        <v>16</v>
-      </c>
-      <c r="D26" s="51"/>
-      <c r="E26" s="52"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="85" t="s">
-        <v>17</v>
-      </c>
-      <c r="B27" s="92" t="s">
-        <v>61</v>
-      </c>
-      <c r="C27" s="93"/>
-      <c r="D27" s="94"/>
-      <c r="E27" s="95"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="86" t="s">
-        <v>18</v>
-      </c>
-      <c r="B28" s="96" t="s">
-        <v>60</v>
-      </c>
-      <c r="C28" s="82"/>
-      <c r="D28"/>
-      <c r="E28" s="97"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="86"/>
-      <c r="B29" s="98" t="s">
-        <v>36</v>
-      </c>
-      <c r="C29" s="82"/>
-      <c r="D29"/>
-      <c r="E29" s="97"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" s="86"/>
-      <c r="B30" s="96" t="s">
+      <c r="B54" s="20"/>
+      <c r="C54" s="24"/>
+      <c r="D54" s="21"/>
+      <c r="E54" s="22"/>
+    </row>
+    <row r="55" spans="1:5" s="16" customFormat="1" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="B55" s="20"/>
+      <c r="C55" s="25"/>
+      <c r="D55" s="21"/>
+      <c r="E55" s="22"/>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A56" s="78" t="s">
+        <v>59</v>
+      </c>
+      <c r="B56"/>
+      <c r="C56" s="78"/>
+      <c r="D56" t="s">
+        <v>66</v>
+      </c>
+      <c r="E56"/>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A57" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C57" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="C30" s="82"/>
-      <c r="D30"/>
-      <c r="E30" s="97"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" s="86" t="s">
-        <v>29</v>
-      </c>
-      <c r="B31" s="98" t="s">
-        <v>43</v>
-      </c>
-      <c r="C31" s="82"/>
-      <c r="D31"/>
-      <c r="E31" s="97"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="86"/>
-      <c r="B32" s="98" t="s">
-        <v>38</v>
-      </c>
-      <c r="C32" s="82"/>
-      <c r="D32"/>
-      <c r="E32" s="97"/>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A33" s="86" t="s">
-        <v>39</v>
-      </c>
-      <c r="B33" s="98" t="s">
-        <v>44</v>
-      </c>
-      <c r="C33" s="82"/>
-      <c r="D33"/>
-      <c r="E33" s="97"/>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A34" s="86"/>
-      <c r="B34" s="99"/>
-      <c r="C34" s="100"/>
-      <c r="D34" s="101"/>
-      <c r="E34" s="102"/>
-    </row>
-    <row r="35" spans="1:6" s="14" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
-      <c r="A35" s="58" t="s">
-        <v>9</v>
-      </c>
-      <c r="B35" s="20"/>
-      <c r="C35" s="20"/>
-      <c r="D35" s="20"/>
-      <c r="E35" s="59"/>
-    </row>
-    <row r="36" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="96" t="s">
-        <v>51</v>
-      </c>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
-      <c r="D36" s="20"/>
-      <c r="E36" s="59"/>
-    </row>
-    <row r="37" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="96" t="s">
-        <v>57</v>
-      </c>
-      <c r="B37" s="20"/>
-      <c r="C37" s="20"/>
-      <c r="D37" s="20"/>
-      <c r="E37" s="59"/>
-    </row>
-    <row r="38" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="96" t="s">
-        <v>52</v>
-      </c>
-      <c r="B38" s="20"/>
-      <c r="C38" s="20"/>
-      <c r="D38" s="20"/>
-      <c r="E38" s="59"/>
-    </row>
-    <row r="39" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="96" t="s">
-        <v>40</v>
-      </c>
-      <c r="B39" s="20"/>
-      <c r="C39" s="20"/>
-      <c r="D39" s="20"/>
-      <c r="E39" s="59"/>
-    </row>
-    <row r="40" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="96" t="s">
-        <v>35</v>
-      </c>
-      <c r="B40" s="20"/>
-      <c r="C40" s="20"/>
-      <c r="D40" s="20"/>
-      <c r="E40" s="59"/>
-    </row>
-    <row r="41" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="96" t="s">
-        <v>32</v>
-      </c>
-      <c r="B41" s="20"/>
-      <c r="C41" s="20"/>
-      <c r="D41" s="20"/>
-      <c r="E41" s="59"/>
-    </row>
-    <row r="42" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="96" t="s">
-        <v>33</v>
-      </c>
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
-      <c r="D42" s="20"/>
-      <c r="E42" s="59"/>
-    </row>
-    <row r="43" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="96" t="s">
-        <v>31</v>
-      </c>
-      <c r="B43" s="45"/>
-      <c r="C43" s="20"/>
-      <c r="D43" s="20"/>
-      <c r="E43" s="59"/>
-    </row>
-    <row r="44" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="96" t="s">
-        <v>34</v>
-      </c>
-      <c r="B44" s="45"/>
-      <c r="C44" s="20"/>
-      <c r="D44" s="20"/>
-      <c r="E44" s="59"/>
-    </row>
-    <row r="45" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="106" t="s">
-        <v>12</v>
-      </c>
-      <c r="B45" s="45"/>
-      <c r="C45" s="20"/>
-      <c r="D45" s="20"/>
-      <c r="E45" s="59"/>
-    </row>
-    <row r="46" spans="1:6" s="14" customFormat="1" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A46" s="104" t="s">
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A58" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B46" s="100"/>
-      <c r="C46" s="100"/>
-      <c r="D46" s="100"/>
-      <c r="E46" s="105"/>
-      <c r="F46" s="103"/>
-    </row>
-    <row r="47" spans="1:6" s="17" customFormat="1" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="54" t="s">
-        <v>27</v>
-      </c>
-      <c r="B47" s="55"/>
-      <c r="C47" s="55"/>
-      <c r="D47" s="56"/>
-      <c r="E47" s="57"/>
-    </row>
-    <row r="48" spans="1:6" s="17" customFormat="1" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="B48" s="22"/>
-      <c r="C48" s="25"/>
-      <c r="D48" s="23"/>
-      <c r="E48" s="24"/>
-    </row>
-    <row r="49" spans="1:5" s="17" customFormat="1" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="B49" s="22"/>
-      <c r="C49" s="26"/>
-      <c r="D49" s="23"/>
-      <c r="E49" s="24"/>
-    </row>
-    <row r="50" spans="1:5" s="17" customFormat="1" ht="18.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B50" s="22"/>
-      <c r="C50" s="26"/>
-      <c r="D50" s="23"/>
-      <c r="E50" s="24"/>
-    </row>
-    <row r="51" spans="1:5" s="17" customFormat="1" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="B51" s="22"/>
-      <c r="C51" s="27"/>
-      <c r="D51" s="23"/>
-      <c r="E51" s="24"/>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A52" s="82" t="s">
-        <v>58</v>
-      </c>
-      <c r="B52"/>
-      <c r="C52" s="82"/>
-      <c r="D52" t="s">
-        <v>67</v>
-      </c>
-      <c r="E52"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A53" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C53" s="18" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A54" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B54" s="8"/>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A55" s="18" t="s">
-        <v>75</v>
-      </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="/O0SEc/iSmo1e/w2Y6a8DFb8iMFyuPCcnw+0QyA4fD0hu1PHUh9xSgVBjmSb8t+GcHdikIUY+NHkooIPanGqkA==" saltValue="RdUcSyAN0Jfo3WDy9ofnyg==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="6N+afjBeGnQ019rumyG/tj7Mw/IbfOJBibcp9bzQlt2/LQ5QJo44vLeSlXXXUBgO7gzIkWMEbDqlERQMsNxGVA==" saltValue="cBuapYocazD4xKlrex10FA==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1"/>
+  <mergeCells count="1">
+    <mergeCell ref="A50:E50"/>
+  </mergeCells>
   <phoneticPr fontId="19" type="noConversion"/>
   <printOptions gridLines="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1916,28 +1952,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="68c6eb59-c8cb-4041-b722-6c1a04bb05c6" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9cd1c65f-f088-4d7a-9266-6a743de4b1cc">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A2D7F59DAA03243959148C4D9985E31" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="41e823b893f608a554722e3854d5a361">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9cd1c65f-f088-4d7a-9266-6a743de4b1cc" xmlns:ns3="68c6eb59-c8cb-4041-b722-6c1a04bb05c6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cbc1271608b89159470addf84b20f7ff" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A2D7F59DAA03243959148C4D9985E31" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="dabbb4365962b50875e117d2bfc07ca0">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9cd1c65f-f088-4d7a-9266-6a743de4b1cc" xmlns:ns3="68c6eb59-c8cb-4041-b722-6c1a04bb05c6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a4ee2e1e860036f5d4feae96d06e8b20" ns2:_="" ns3:_="">
     <xsd:import namespace="9cd1c65f-f088-4d7a-9266-6a743de4b1cc"/>
     <xsd:import namespace="68c6eb59-c8cb-4041-b722-6c1a04bb05c6"/>
     <xsd:element name="properties">
@@ -1958,6 +1974,8 @@
                 <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
                 <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
                 <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -2015,6 +2033,16 @@
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
         </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="21" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="22" nillable="true" ma:displayName="Location" ma:description="" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -2158,27 +2186,28 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C63E2DBE-5738-4463-A2C9-8D3B6BAF2444}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="68c6eb59-c8cb-4041-b722-6c1a04bb05c6"/>
-    <ds:schemaRef ds:uri="9cd1c65f-f088-4d7a-9266-6a743de4b1cc"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="68c6eb59-c8cb-4041-b722-6c1a04bb05c6" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9cd1c65f-f088-4d7a-9266-6a743de4b1cc">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17D82BCE-1C07-45EA-A14B-B1392CD4B9CA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC8E1665-2065-41B4-B13F-EF7809DFCCE5}">
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23131BE1-8C5C-4D85-B362-63EF2C751404}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
@@ -2194,4 +2223,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22040A60-7C10-4D1E-8A7F-B2A25CD99515}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="68c6eb59-c8cb-4041-b722-6c1a04bb05c6"/>
+    <ds:schemaRef ds:uri="9cd1c65f-f088-4d7a-9266-6a743de4b1cc"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8240839-31BF-4102-B13C-17B3AA02EE33}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>